<commit_message>
correct some paths in scripts
</commit_message>
<xml_diff>
--- a/data/spermidine_exp_data.xlsx
+++ b/data/spermidine_exp_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\github\etfl\ETFLdesigner\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D31D31B-E4B0-41CA-81E3-BA04AA8CE62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5033A5BB-1CF8-4339-B19A-E2E124DF6BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="10215" yWindow="3570" windowWidth="18285" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -581,6 +581,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H24"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="16.25" customWidth="1"/>
+    <col min="5" max="5" width="14.625" customWidth="1"/>
+    <col min="6" max="6" width="18.875" customWidth="1"/>
+    <col min="7" max="7" width="24.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">

</xml_diff>